<commit_message>
L1 permutations 100 50 1B
</commit_message>
<xml_diff>
--- a/data/sim_status.xlsx
+++ b/data/sim_status.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/emilio.lopez/code_repos/investigacion/publicaciones/fda-monitoring-framework/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1355E5B7-1074-4044-8AA0-E3988B8CB933}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D2E4168-EE01-F045-B6AC-B5FD4FD8399F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="520" yWindow="800" windowWidth="14800" windowHeight="17180" xr2:uid="{A288BA06-CF39-B046-86D3-43E918745413}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="405" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="409" uniqueCount="155">
   <si>
     <t>l1std_bootstrap_100_50_1A.R</t>
   </si>
@@ -1399,10 +1399,10 @@
       </c>
       <c r="C30" s="2"/>
       <c r="D30" t="s">
-        <v>135</v>
+        <v>121</v>
       </c>
       <c r="F30" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.2">
@@ -1472,6 +1472,13 @@
       <c r="B35" t="s">
         <v>40</v>
       </c>
+      <c r="C35" s="1"/>
+      <c r="D35" t="s">
+        <v>117</v>
+      </c>
+      <c r="F35" t="s">
+        <v>120</v>
+      </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
@@ -1479,6 +1486,13 @@
       </c>
       <c r="B36" t="s">
         <v>41</v>
+      </c>
+      <c r="C36" s="2"/>
+      <c r="D36" t="s">
+        <v>117</v>
+      </c>
+      <c r="F36" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
l1 permutations 150 100 1B
</commit_message>
<xml_diff>
--- a/data/sim_status.xlsx
+++ b/data/sim_status.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/emilio.lopez/code_repos/investigacion/publicaciones/fda-monitoring-framework/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D2E4168-EE01-F045-B6AC-B5FD4FD8399F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18E7B99D-50AD-E548-A02D-499BFCB7EE25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="520" yWindow="800" windowWidth="14800" windowHeight="17180" xr2:uid="{A288BA06-CF39-B046-86D3-43E918745413}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="409" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="156">
   <si>
     <t>l1std_bootstrap_100_50_1A.R</t>
   </si>
@@ -504,6 +504,9 @@
   </si>
   <si>
     <t>1.16 days</t>
+  </si>
+  <si>
+    <t>17 hours</t>
   </si>
 </sst>
 </file>
@@ -1397,9 +1400,12 @@
       <c r="B30" t="s">
         <v>35</v>
       </c>
-      <c r="C30" s="2"/>
+      <c r="C30" s="1"/>
       <c r="D30" t="s">
         <v>121</v>
+      </c>
+      <c r="E30" t="s">
+        <v>155</v>
       </c>
       <c r="F30" t="s">
         <v>122</v>
@@ -1487,7 +1493,7 @@
       <c r="B36" t="s">
         <v>41</v>
       </c>
-      <c r="C36" s="2"/>
+      <c r="C36" s="1"/>
       <c r="D36" t="s">
         <v>117</v>
       </c>
@@ -1502,6 +1508,13 @@
       <c r="B37" t="s">
         <v>42</v>
       </c>
+      <c r="C37" s="2"/>
+      <c r="D37" t="s">
+        <v>133</v>
+      </c>
+      <c r="F37" t="s">
+        <v>122</v>
+      </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
@@ -1509,6 +1522,13 @@
       </c>
       <c r="B38" t="s">
         <v>43</v>
+      </c>
+      <c r="C38" s="2"/>
+      <c r="D38" t="s">
+        <v>117</v>
+      </c>
+      <c r="F38" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
L2 bootstrap 150 100 1B
</commit_message>
<xml_diff>
--- a/data/sim_status.xlsx
+++ b/data/sim_status.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/emilio.lopez/code_repos/investigacion/publicaciones/fda-monitoring-framework/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18E7B99D-50AD-E548-A02D-499BFCB7EE25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE52E816-3E18-8340-BE31-1680D7CCBE0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="520" yWindow="800" windowWidth="14800" windowHeight="17180" xr2:uid="{A288BA06-CF39-B046-86D3-43E918745413}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="156">
   <si>
     <t>l1std_bootstrap_100_50_1A.R</t>
   </si>
@@ -1523,7 +1523,7 @@
       <c r="B38" t="s">
         <v>43</v>
       </c>
-      <c r="C38" s="2"/>
+      <c r="C38" s="1"/>
       <c r="D38" t="s">
         <v>117</v>
       </c>
@@ -1538,6 +1538,13 @@
       <c r="B39" t="s">
         <v>44</v>
       </c>
+      <c r="C39" s="1"/>
+      <c r="D39" t="s">
+        <v>117</v>
+      </c>
+      <c r="F39" t="s">
+        <v>120</v>
+      </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
@@ -1545,6 +1552,13 @@
       </c>
       <c r="B40" t="s">
         <v>45</v>
+      </c>
+      <c r="C40" s="2"/>
+      <c r="D40" t="s">
+        <v>117</v>
+      </c>
+      <c r="F40" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.2">
@@ -1716,7 +1730,10 @@
       <c r="B56" t="s">
         <v>62</v>
       </c>
-      <c r="C56" s="2"/>
+      <c r="C56" s="1"/>
+      <c r="F56" t="s">
+        <v>126</v>
+      </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
@@ -1734,7 +1751,10 @@
       <c r="B58" t="s">
         <v>64</v>
       </c>
-      <c r="C58" s="2"/>
+      <c r="C58" s="1"/>
+      <c r="F58" t="s">
+        <v>126</v>
+      </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
@@ -1806,7 +1826,10 @@
       <c r="B64" t="s">
         <v>70</v>
       </c>
-      <c r="C64" s="2"/>
+      <c r="C64" s="1"/>
+      <c r="F64" t="s">
+        <v>126</v>
+      </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
@@ -1815,7 +1838,7 @@
       <c r="B65" t="s">
         <v>71</v>
       </c>
-      <c r="C65" s="2"/>
+      <c r="C65" s="1"/>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
@@ -1824,7 +1847,10 @@
       <c r="B66" t="s">
         <v>72</v>
       </c>
-      <c r="C66" s="2"/>
+      <c r="C66" s="1"/>
+      <c r="F66" t="s">
+        <v>126</v>
+      </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
@@ -1833,7 +1859,10 @@
       <c r="B67" t="s">
         <v>73</v>
       </c>
-      <c r="C67" s="2"/>
+      <c r="C67" s="1"/>
+      <c r="F67" t="s">
+        <v>126</v>
+      </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
@@ -1908,7 +1937,10 @@
       <c r="B73" t="s">
         <v>79</v>
       </c>
-      <c r="C73" s="2"/>
+      <c r="C73" s="1"/>
+      <c r="F73" t="s">
+        <v>126</v>
+      </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
@@ -1917,7 +1949,10 @@
       <c r="B74" t="s">
         <v>80</v>
       </c>
-      <c r="C74" s="2"/>
+      <c r="C74" s="1"/>
+      <c r="F74" t="s">
+        <v>126</v>
+      </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
@@ -1926,7 +1961,10 @@
       <c r="B75" t="s">
         <v>81</v>
       </c>
-      <c r="C75" s="2"/>
+      <c r="C75" s="1"/>
+      <c r="F75" t="s">
+        <v>126</v>
+      </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
@@ -1935,7 +1973,10 @@
       <c r="B76" t="s">
         <v>82</v>
       </c>
-      <c r="C76" s="2"/>
+      <c r="C76" s="1"/>
+      <c r="F76" t="s">
+        <v>126</v>
+      </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
@@ -1989,7 +2030,10 @@
       <c r="B80" t="s">
         <v>86</v>
       </c>
-      <c r="C80" s="2"/>
+      <c r="C80" s="1"/>
+      <c r="F80" t="s">
+        <v>126</v>
+      </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
@@ -2007,7 +2051,10 @@
       <c r="B82" t="s">
         <v>88</v>
       </c>
-      <c r="C82" s="2"/>
+      <c r="C82" s="1"/>
+      <c r="F82" t="s">
+        <v>126</v>
+      </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A83" t="s">

</xml_diff>

<commit_message>
L2 bootstrap 200 100 1B
</commit_message>
<xml_diff>
--- a/data/sim_status.xlsx
+++ b/data/sim_status.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/emilio.lopez/code_repos/investigacion/publicaciones/fda-monitoring-framework/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE52E816-3E18-8340-BE31-1680D7CCBE0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A642E48F-C087-304F-8B60-F3D712D13489}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="520" yWindow="800" windowWidth="14800" windowHeight="17180" xr2:uid="{A288BA06-CF39-B046-86D3-43E918745413}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="438" uniqueCount="157">
   <si>
     <t>l1std_bootstrap_100_50_1A.R</t>
   </si>
@@ -507,6 +507,9 @@
   </si>
   <si>
     <t>17 hours</t>
+  </si>
+  <si>
+    <t>4,5 days</t>
   </si>
 </sst>
 </file>
@@ -1418,9 +1421,12 @@
       <c r="B31" t="s">
         <v>36</v>
       </c>
-      <c r="C31" s="2"/>
+      <c r="C31" s="1"/>
       <c r="D31" t="s">
         <v>125</v>
+      </c>
+      <c r="E31" t="s">
+        <v>156</v>
       </c>
       <c r="F31" t="s">
         <v>120</v>
@@ -1508,7 +1514,7 @@
       <c r="B37" t="s">
         <v>42</v>
       </c>
-      <c r="C37" s="2"/>
+      <c r="C37" s="1"/>
       <c r="D37" t="s">
         <v>133</v>
       </c>
@@ -1553,7 +1559,7 @@
       <c r="B40" t="s">
         <v>45</v>
       </c>
-      <c r="C40" s="2"/>
+      <c r="C40" s="1"/>
       <c r="D40" t="s">
         <v>117</v>
       </c>
@@ -1613,6 +1619,13 @@
       <c r="B44" t="s">
         <v>49</v>
       </c>
+      <c r="C44" s="2"/>
+      <c r="D44" t="s">
+        <v>117</v>
+      </c>
+      <c r="F44" t="s">
+        <v>120</v>
+      </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
@@ -1637,6 +1650,13 @@
       <c r="B47" t="s">
         <v>52</v>
       </c>
+      <c r="C47" s="1"/>
+      <c r="D47" t="s">
+        <v>133</v>
+      </c>
+      <c r="F47" t="s">
+        <v>122</v>
+      </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
@@ -1645,6 +1665,13 @@
       <c r="B48" t="s">
         <v>53</v>
       </c>
+      <c r="C48" s="2"/>
+      <c r="D48" t="s">
+        <v>125</v>
+      </c>
+      <c r="F48" t="s">
+        <v>120</v>
+      </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
@@ -1652,6 +1679,13 @@
       </c>
       <c r="B49" t="s">
         <v>54</v>
+      </c>
+      <c r="C49" s="2"/>
+      <c r="D49" t="s">
+        <v>133</v>
+      </c>
+      <c r="F49" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
L2 permutations 100 50 1B
</commit_message>
<xml_diff>
--- a/data/sim_status.xlsx
+++ b/data/sim_status.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/emilio.lopez/code_repos/investigacion/publicaciones/fda-monitoring-framework/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A642E48F-C087-304F-8B60-F3D712D13489}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89A5F9B0-DC20-A248-8E5F-152107F9E6DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="520" yWindow="800" windowWidth="14800" windowHeight="17180" xr2:uid="{A288BA06-CF39-B046-86D3-43E918745413}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="438" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="440" uniqueCount="157">
   <si>
     <t>l1std_bootstrap_100_50_1A.R</t>
   </si>
@@ -1619,7 +1619,7 @@
       <c r="B44" t="s">
         <v>49</v>
       </c>
-      <c r="C44" s="2"/>
+      <c r="C44" s="1"/>
       <c r="D44" t="s">
         <v>117</v>
       </c>
@@ -1633,6 +1633,13 @@
       </c>
       <c r="B45" t="s">
         <v>50</v>
+      </c>
+      <c r="C45" s="2"/>
+      <c r="D45" t="s">
+        <v>117</v>
+      </c>
+      <c r="F45" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
L2 permutations 150 100 1B
</commit_message>
<xml_diff>
--- a/data/sim_status.xlsx
+++ b/data/sim_status.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/emilio.lopez/code_repos/investigacion/publicaciones/fda-monitoring-framework/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89A5F9B0-DC20-A248-8E5F-152107F9E6DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A89F5ED-D6B5-3645-92D2-D2235BEF1B10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="520" yWindow="800" windowWidth="14800" windowHeight="17180" xr2:uid="{A288BA06-CF39-B046-86D3-43E918745413}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="440" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="443" uniqueCount="158">
   <si>
     <t>l1std_bootstrap_100_50_1A.R</t>
   </si>
@@ -510,6 +510,9 @@
   </si>
   <si>
     <t>4,5 days</t>
+  </si>
+  <si>
+    <t>13.4 hours</t>
   </si>
 </sst>
 </file>
@@ -1634,10 +1637,13 @@
       <c r="B45" t="s">
         <v>50</v>
       </c>
-      <c r="C45" s="2"/>
+      <c r="C45" s="1"/>
       <c r="D45" t="s">
         <v>117</v>
       </c>
+      <c r="E45" t="s">
+        <v>157</v>
+      </c>
       <c r="F45" t="s">
         <v>120</v>
       </c>
@@ -1648,6 +1654,13 @@
       </c>
       <c r="B46" t="s">
         <v>51</v>
+      </c>
+      <c r="C46" s="2"/>
+      <c r="D46" t="s">
+        <v>117</v>
+      </c>
+      <c r="F46" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
L2 permutations 200 100 1B
</commit_message>
<xml_diff>
--- a/data/sim_status.xlsx
+++ b/data/sim_status.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/emilio.lopez/code_repos/investigacion/publicaciones/fda-monitoring-framework/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A89F5ED-D6B5-3645-92D2-D2235BEF1B10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15E273E1-1E4A-5946-B6EE-D63655F3FD52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="520" yWindow="800" windowWidth="14800" windowHeight="17180" xr2:uid="{A288BA06-CF39-B046-86D3-43E918745413}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="443" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="455" uniqueCount="161">
   <si>
     <t>l1std_bootstrap_100_50_1A.R</t>
   </si>
@@ -513,6 +513,15 @@
   </si>
   <si>
     <t>13.4 hours</t>
+  </si>
+  <si>
+    <t>1,21 days</t>
+  </si>
+  <si>
+    <t>8,88 hours</t>
+  </si>
+  <si>
+    <t>22,7 hours</t>
   </si>
 </sst>
 </file>
@@ -1655,9 +1664,12 @@
       <c r="B46" t="s">
         <v>51</v>
       </c>
-      <c r="C46" s="2"/>
+      <c r="C46" s="1"/>
       <c r="D46" t="s">
         <v>117</v>
+      </c>
+      <c r="E46" t="s">
+        <v>160</v>
       </c>
       <c r="F46" t="s">
         <v>120</v>
@@ -1700,9 +1712,12 @@
       <c r="B49" t="s">
         <v>54</v>
       </c>
-      <c r="C49" s="2"/>
+      <c r="C49" s="1"/>
       <c r="D49" t="s">
         <v>133</v>
+      </c>
+      <c r="E49" t="s">
+        <v>158</v>
       </c>
       <c r="F49" t="s">
         <v>122</v>
@@ -1760,6 +1775,16 @@
       <c r="B53" t="s">
         <v>58</v>
       </c>
+      <c r="C53" s="1"/>
+      <c r="D53" t="s">
+        <v>133</v>
+      </c>
+      <c r="E53" t="s">
+        <v>159</v>
+      </c>
+      <c r="F53" t="s">
+        <v>122</v>
+      </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
@@ -1768,6 +1793,13 @@
       <c r="B54" t="s">
         <v>59</v>
       </c>
+      <c r="C54" s="2"/>
+      <c r="D54" t="s">
+        <v>133</v>
+      </c>
+      <c r="F54" t="s">
+        <v>122</v>
+      </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
@@ -1776,6 +1808,13 @@
       <c r="B55" t="s">
         <v>60</v>
       </c>
+      <c r="C55" s="2"/>
+      <c r="D55" t="s">
+        <v>117</v>
+      </c>
+      <c r="F55" t="s">
+        <v>120</v>
+      </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
@@ -1796,7 +1835,10 @@
       <c r="B57" t="s">
         <v>63</v>
       </c>
-      <c r="C57" s="2"/>
+      <c r="C57" s="1"/>
+      <c r="F57" t="s">
+        <v>126</v>
+      </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
@@ -1982,7 +2024,10 @@
       <c r="B72" t="s">
         <v>78</v>
       </c>
-      <c r="C72" s="2"/>
+      <c r="C72" s="1"/>
+      <c r="F72" t="s">
+        <v>126</v>
+      </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
@@ -2096,7 +2141,10 @@
       <c r="B81" t="s">
         <v>87</v>
       </c>
-      <c r="C81" s="2"/>
+      <c r="C81" s="1"/>
+      <c r="F81" t="s">
+        <v>126</v>
+      </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A82" t="s">

</xml_diff>

<commit_message>
T2 permutations 200 100 1B
</commit_message>
<xml_diff>
--- a/data/sim_status.xlsx
+++ b/data/sim_status.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/emilio.lopez/code_repos/investigacion/publicaciones/fda-monitoring-framework/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15E273E1-1E4A-5946-B6EE-D63655F3FD52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56B5B119-8731-6E42-AFF0-276918F81FFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="520" yWindow="800" windowWidth="14800" windowHeight="17180" xr2:uid="{A288BA06-CF39-B046-86D3-43E918745413}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="455" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="456" uniqueCount="161">
   <si>
     <t>l1std_bootstrap_100_50_1A.R</t>
   </si>
@@ -1913,7 +1913,10 @@
       <c r="B63" t="s">
         <v>69</v>
       </c>
-      <c r="C63" s="2"/>
+      <c r="C63" s="1"/>
+      <c r="F63" t="s">
+        <v>126</v>
+      </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A64" t="s">

</xml_diff>

<commit_message>
L1 permutations 2A missing
</commit_message>
<xml_diff>
--- a/data/sim_status.xlsx
+++ b/data/sim_status.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/emilio.lopez/code_repos/investigacion/publicaciones/fda-monitoring-framework/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56B5B119-8731-6E42-AFF0-276918F81FFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC8C0899-06B1-D94E-BB20-3DCA62163CFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="520" yWindow="800" windowWidth="14800" windowHeight="17180" xr2:uid="{A288BA06-CF39-B046-86D3-43E918745413}"/>
+    <workbookView xWindow="6420" yWindow="1080" windowWidth="14800" windowHeight="17180" xr2:uid="{A288BA06-CF39-B046-86D3-43E918745413}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="456" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="462" uniqueCount="164">
   <si>
     <t>l1std_bootstrap_100_50_1A.R</t>
   </si>
@@ -522,6 +522,15 @@
   </si>
   <si>
     <t>22,7 hours</t>
+  </si>
+  <si>
+    <t>3 days</t>
+  </si>
+  <si>
+    <t>24 hours</t>
+  </si>
+  <si>
+    <t>M4</t>
   </si>
 </sst>
 </file>
@@ -537,7 +546,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -556,6 +565,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -569,10 +584,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -916,22 +933,17 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B1" t="s">
-        <v>29</v>
-      </c>
-      <c r="C1" t="s">
-        <v>31</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="C1" s="1"/>
       <c r="D1" t="s">
-        <v>32</v>
-      </c>
-      <c r="E1" t="s">
-        <v>33</v>
+        <v>117</v>
       </c>
       <c r="F1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>127</v>
@@ -942,7 +954,7 @@
         <v>28</v>
       </c>
       <c r="B2" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" t="s">
@@ -960,7 +972,7 @@
         <v>28</v>
       </c>
       <c r="B3" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C3" s="1"/>
       <c r="D3" t="s">
@@ -975,11 +987,11 @@
         <v>28</v>
       </c>
       <c r="B4" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C4" s="1"/>
       <c r="D4" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="F4" t="s">
         <v>120</v>
@@ -990,7 +1002,7 @@
         <v>28</v>
       </c>
       <c r="B5" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C5" s="1"/>
       <c r="D5" t="s">
@@ -1005,7 +1017,7 @@
         <v>28</v>
       </c>
       <c r="B6" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C6" s="1"/>
       <c r="D6" t="s">
@@ -1020,14 +1032,17 @@
         <v>28</v>
       </c>
       <c r="B7" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C7" s="1"/>
       <c r="D7" t="s">
-        <v>125</v>
+        <v>121</v>
+      </c>
+      <c r="E7" t="s">
+        <v>124</v>
       </c>
       <c r="F7" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
@@ -1035,14 +1050,14 @@
         <v>28</v>
       </c>
       <c r="B8" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C8" s="1"/>
       <c r="D8" t="s">
         <v>121</v>
       </c>
       <c r="E8" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F8" t="s">
         <v>122</v>
@@ -1053,14 +1068,14 @@
         <v>28</v>
       </c>
       <c r="B9" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C9" s="1"/>
       <c r="D9" t="s">
         <v>121</v>
       </c>
       <c r="E9" t="s">
-        <v>123</v>
+        <v>130</v>
       </c>
       <c r="F9" t="s">
         <v>122</v>
@@ -1071,17 +1086,17 @@
         <v>28</v>
       </c>
       <c r="B10" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C10" s="1"/>
       <c r="D10" t="s">
-        <v>121</v>
+        <v>136</v>
       </c>
       <c r="E10" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="F10" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
@@ -1089,14 +1104,14 @@
         <v>28</v>
       </c>
       <c r="B11" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C11" s="1"/>
       <c r="D11" t="s">
         <v>136</v>
       </c>
       <c r="E11" t="s">
-        <v>124</v>
+        <v>137</v>
       </c>
       <c r="F11" t="s">
         <v>126</v>
@@ -1107,14 +1122,14 @@
         <v>28</v>
       </c>
       <c r="B12" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C12" s="1"/>
       <c r="D12" t="s">
         <v>136</v>
       </c>
       <c r="E12" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="F12" t="s">
         <v>126</v>
@@ -1125,17 +1140,14 @@
         <v>28</v>
       </c>
       <c r="B13" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C13" s="1"/>
       <c r="D13" t="s">
-        <v>136</v>
-      </c>
-      <c r="E13" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="F13" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
@@ -1143,7 +1155,7 @@
         <v>28</v>
       </c>
       <c r="B14" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C14" s="1"/>
       <c r="D14" t="s">
@@ -1158,7 +1170,7 @@
         <v>28</v>
       </c>
       <c r="B15" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C15" s="1"/>
       <c r="D15" t="s">
@@ -1173,11 +1185,14 @@
         <v>28</v>
       </c>
       <c r="B16" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C16" s="1"/>
       <c r="D16" t="s">
-        <v>125</v>
+        <v>117</v>
+      </c>
+      <c r="E16" t="s">
+        <v>118</v>
       </c>
       <c r="F16" t="s">
         <v>120</v>
@@ -1188,14 +1203,14 @@
         <v>28</v>
       </c>
       <c r="B17" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C17" s="1"/>
       <c r="D17" t="s">
         <v>117</v>
       </c>
       <c r="E17" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="F17" t="s">
         <v>120</v>
@@ -1206,14 +1221,14 @@
         <v>28</v>
       </c>
       <c r="B18" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C18" s="1"/>
       <c r="D18" t="s">
         <v>117</v>
       </c>
       <c r="E18" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="F18" t="s">
         <v>120</v>
@@ -1224,17 +1239,17 @@
         <v>28</v>
       </c>
       <c r="B19" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C19" s="1"/>
       <c r="D19" t="s">
-        <v>117</v>
+        <v>136</v>
       </c>
       <c r="E19" t="s">
         <v>131</v>
       </c>
       <c r="F19" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.2">
@@ -1242,14 +1257,14 @@
         <v>28</v>
       </c>
       <c r="B20" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C20" s="1"/>
       <c r="D20" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="E20" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="F20" t="s">
         <v>126</v>
@@ -1260,14 +1275,14 @@
         <v>28</v>
       </c>
       <c r="B21" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C21" s="1"/>
       <c r="D21" t="s">
         <v>138</v>
       </c>
       <c r="E21" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F21" t="s">
         <v>126</v>
@@ -1278,17 +1293,14 @@
         <v>28</v>
       </c>
       <c r="B22" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C22" s="1"/>
       <c r="D22" t="s">
-        <v>138</v>
-      </c>
-      <c r="E22" t="s">
-        <v>140</v>
+        <v>125</v>
       </c>
       <c r="F22" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.2">
@@ -1296,7 +1308,7 @@
         <v>28</v>
       </c>
       <c r="B23" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C23" s="1"/>
       <c r="D23" t="s">
@@ -1311,7 +1323,7 @@
         <v>28</v>
       </c>
       <c r="B24" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C24" s="1"/>
       <c r="D24" t="s">
@@ -1326,14 +1338,17 @@
         <v>28</v>
       </c>
       <c r="B25" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C25" s="1"/>
       <c r="D25" t="s">
-        <v>125</v>
+        <v>133</v>
+      </c>
+      <c r="E25" t="s">
+        <v>134</v>
       </c>
       <c r="F25" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.2">
@@ -1341,14 +1356,14 @@
         <v>28</v>
       </c>
       <c r="B26" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C26" s="1"/>
       <c r="D26" t="s">
-        <v>133</v>
+        <v>121</v>
       </c>
       <c r="E26" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="F26" t="s">
         <v>122</v>
@@ -1359,32 +1374,32 @@
         <v>28</v>
       </c>
       <c r="B27" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C27" s="1"/>
       <c r="D27" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="E27" t="s">
-        <v>131</v>
+        <v>154</v>
       </c>
       <c r="F27" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B28" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="C28" s="1"/>
       <c r="D28" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="E28" t="s">
-        <v>154</v>
+        <v>132</v>
       </c>
       <c r="F28" t="s">
         <v>120</v>
@@ -1395,17 +1410,17 @@
         <v>30</v>
       </c>
       <c r="B29" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C29" s="1"/>
       <c r="D29" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="E29" t="s">
-        <v>132</v>
+        <v>155</v>
       </c>
       <c r="F29" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.2">
@@ -1413,17 +1428,17 @@
         <v>30</v>
       </c>
       <c r="B30" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C30" s="1"/>
       <c r="D30" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="E30" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F30" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.2">
@@ -1431,15 +1446,12 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C31" s="1"/>
       <c r="D31" t="s">
         <v>125</v>
       </c>
-      <c r="E31" t="s">
-        <v>156</v>
-      </c>
       <c r="F31" t="s">
         <v>120</v>
       </c>
@@ -1449,7 +1461,7 @@
         <v>30</v>
       </c>
       <c r="B32" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C32" s="1"/>
       <c r="D32" t="s">
@@ -1464,7 +1476,7 @@
         <v>30</v>
       </c>
       <c r="B33" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C33" s="1"/>
       <c r="D33" t="s">
@@ -1479,11 +1491,11 @@
         <v>30</v>
       </c>
       <c r="B34" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C34" s="1"/>
       <c r="D34" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="F34" t="s">
         <v>120</v>
@@ -1494,7 +1506,7 @@
         <v>30</v>
       </c>
       <c r="B35" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C35" s="1"/>
       <c r="D35" t="s">
@@ -1509,14 +1521,14 @@
         <v>30</v>
       </c>
       <c r="B36" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C36" s="1"/>
       <c r="D36" t="s">
-        <v>117</v>
+        <v>133</v>
       </c>
       <c r="F36" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.2">
@@ -1524,14 +1536,14 @@
         <v>30</v>
       </c>
       <c r="B37" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C37" s="1"/>
       <c r="D37" t="s">
-        <v>133</v>
+        <v>117</v>
       </c>
       <c r="F37" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.2">
@@ -1539,7 +1551,7 @@
         <v>30</v>
       </c>
       <c r="B38" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C38" s="1"/>
       <c r="D38" t="s">
@@ -1554,7 +1566,7 @@
         <v>30</v>
       </c>
       <c r="B39" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C39" s="1"/>
       <c r="D39" t="s">
@@ -1569,11 +1581,11 @@
         <v>30</v>
       </c>
       <c r="B40" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C40" s="1"/>
       <c r="D40" t="s">
-        <v>117</v>
+        <v>135</v>
       </c>
       <c r="F40" t="s">
         <v>120</v>
@@ -1584,7 +1596,7 @@
         <v>30</v>
       </c>
       <c r="B41" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C41" s="1"/>
       <c r="D41" t="s">
@@ -1599,7 +1611,7 @@
         <v>30</v>
       </c>
       <c r="B42" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C42" s="1"/>
       <c r="D42" t="s">
@@ -1614,11 +1626,11 @@
         <v>30</v>
       </c>
       <c r="B43" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C43" s="1"/>
       <c r="D43" t="s">
-        <v>135</v>
+        <v>117</v>
       </c>
       <c r="F43" t="s">
         <v>120</v>
@@ -1629,12 +1641,15 @@
         <v>30</v>
       </c>
       <c r="B44" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C44" s="1"/>
       <c r="D44" t="s">
         <v>117</v>
       </c>
+      <c r="E44" t="s">
+        <v>157</v>
+      </c>
       <c r="F44" t="s">
         <v>120</v>
       </c>
@@ -1644,14 +1659,14 @@
         <v>30</v>
       </c>
       <c r="B45" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C45" s="1"/>
       <c r="D45" t="s">
         <v>117</v>
       </c>
       <c r="E45" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="F45" t="s">
         <v>120</v>
@@ -1662,17 +1677,14 @@
         <v>30</v>
       </c>
       <c r="B46" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C46" s="1"/>
       <c r="D46" t="s">
-        <v>117</v>
-      </c>
-      <c r="E46" t="s">
-        <v>160</v>
+        <v>133</v>
       </c>
       <c r="F46" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.2">
@@ -1680,14 +1692,17 @@
         <v>30</v>
       </c>
       <c r="B47" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C47" s="1"/>
       <c r="D47" t="s">
-        <v>133</v>
+        <v>125</v>
+      </c>
+      <c r="E47" t="s">
+        <v>161</v>
       </c>
       <c r="F47" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.2">
@@ -1695,14 +1710,17 @@
         <v>30</v>
       </c>
       <c r="B48" t="s">
-        <v>53</v>
-      </c>
-      <c r="C48" s="2"/>
+        <v>54</v>
+      </c>
+      <c r="C48" s="1"/>
       <c r="D48" t="s">
-        <v>125</v>
+        <v>133</v>
+      </c>
+      <c r="E48" t="s">
+        <v>158</v>
       </c>
       <c r="F48" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.2">
@@ -1710,17 +1728,14 @@
         <v>30</v>
       </c>
       <c r="B49" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C49" s="1"/>
       <c r="D49" t="s">
-        <v>133</v>
-      </c>
-      <c r="E49" t="s">
-        <v>158</v>
+        <v>135</v>
       </c>
       <c r="F49" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.2">
@@ -1728,7 +1743,7 @@
         <v>30</v>
       </c>
       <c r="B50" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C50" s="1"/>
       <c r="D50" t="s">
@@ -1743,7 +1758,7 @@
         <v>30</v>
       </c>
       <c r="B51" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C51" s="1"/>
       <c r="D51" t="s">
@@ -1758,14 +1773,17 @@
         <v>30</v>
       </c>
       <c r="B52" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C52" s="1"/>
       <c r="D52" t="s">
-        <v>135</v>
+        <v>133</v>
+      </c>
+      <c r="E52" t="s">
+        <v>159</v>
       </c>
       <c r="F52" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.2">
@@ -1773,15 +1791,12 @@
         <v>30</v>
       </c>
       <c r="B53" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C53" s="1"/>
       <c r="D53" t="s">
         <v>133</v>
       </c>
-      <c r="E53" t="s">
-        <v>159</v>
-      </c>
       <c r="F53" t="s">
         <v>122</v>
       </c>
@@ -1791,29 +1806,29 @@
         <v>30</v>
       </c>
       <c r="B54" t="s">
-        <v>59</v>
-      </c>
-      <c r="C54" s="2"/>
+        <v>60</v>
+      </c>
+      <c r="C54" s="1"/>
       <c r="D54" t="s">
-        <v>133</v>
+        <v>117</v>
+      </c>
+      <c r="E54" t="s">
+        <v>162</v>
       </c>
       <c r="F54" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>30</v>
+        <v>61</v>
       </c>
       <c r="B55" t="s">
-        <v>60</v>
-      </c>
-      <c r="C55" s="2"/>
-      <c r="D55" t="s">
-        <v>117</v>
-      </c>
+        <v>62</v>
+      </c>
+      <c r="C55" s="1"/>
       <c r="F55" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.2">
@@ -1821,7 +1836,7 @@
         <v>61</v>
       </c>
       <c r="B56" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C56" s="1"/>
       <c r="F56" t="s">
@@ -1833,7 +1848,7 @@
         <v>61</v>
       </c>
       <c r="B57" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C57" s="1"/>
       <c r="F57" t="s">
@@ -1844,20 +1859,23 @@
       <c r="A58" t="s">
         <v>61</v>
       </c>
-      <c r="B58" t="s">
-        <v>64</v>
+      <c r="B58" s="4" t="s">
+        <v>65</v>
       </c>
       <c r="C58" s="1"/>
+      <c r="D58" t="s">
+        <v>135</v>
+      </c>
       <c r="F58" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>61</v>
       </c>
-      <c r="B59" t="s">
-        <v>65</v>
+      <c r="B59" s="4" t="s">
+        <v>66</v>
       </c>
       <c r="C59" s="1"/>
       <c r="D59" t="s">
@@ -1871,8 +1889,8 @@
       <c r="A60" t="s">
         <v>61</v>
       </c>
-      <c r="B60" t="s">
-        <v>66</v>
+      <c r="B60" s="4" t="s">
+        <v>67</v>
       </c>
       <c r="C60" s="1"/>
       <c r="D60" t="s">
@@ -1886,12 +1904,12 @@
       <c r="A61" t="s">
         <v>61</v>
       </c>
-      <c r="B61" t="s">
-        <v>67</v>
+      <c r="B61" s="3" t="s">
+        <v>68</v>
       </c>
       <c r="C61" s="1"/>
       <c r="D61" t="s">
-        <v>135</v>
+        <v>163</v>
       </c>
       <c r="F61" t="s">
         <v>120</v>
@@ -1901,17 +1919,23 @@
       <c r="A62" t="s">
         <v>61</v>
       </c>
-      <c r="B62" t="s">
-        <v>68</v>
+      <c r="B62" s="3" t="s">
+        <v>69</v>
       </c>
       <c r="C62" s="2"/>
+      <c r="D62" t="s">
+        <v>163</v>
+      </c>
+      <c r="F62" t="s">
+        <v>120</v>
+      </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>61</v>
       </c>
       <c r="B63" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C63" s="1"/>
       <c r="F63" t="s">
@@ -1923,7 +1947,7 @@
         <v>61</v>
       </c>
       <c r="B64" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C64" s="1"/>
       <c r="F64" t="s">
@@ -1935,16 +1959,19 @@
         <v>61</v>
       </c>
       <c r="B65" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C65" s="1"/>
+      <c r="F65" t="s">
+        <v>126</v>
+      </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>61</v>
       </c>
       <c r="B66" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C66" s="1"/>
       <c r="F66" t="s">
@@ -1955,20 +1982,23 @@
       <c r="A67" t="s">
         <v>61</v>
       </c>
-      <c r="B67" t="s">
-        <v>73</v>
+      <c r="B67" s="4" t="s">
+        <v>74</v>
       </c>
       <c r="C67" s="1"/>
+      <c r="D67" t="s">
+        <v>135</v>
+      </c>
       <c r="F67" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>61</v>
       </c>
-      <c r="B68" t="s">
-        <v>74</v>
+      <c r="B68" s="4" t="s">
+        <v>75</v>
       </c>
       <c r="C68" s="1"/>
       <c r="D68" t="s">
@@ -1982,8 +2012,8 @@
       <c r="A69" t="s">
         <v>61</v>
       </c>
-      <c r="B69" t="s">
-        <v>75</v>
+      <c r="B69" s="4" t="s">
+        <v>76</v>
       </c>
       <c r="C69" s="1"/>
       <c r="D69" t="s">
@@ -1998,14 +2028,11 @@
         <v>61</v>
       </c>
       <c r="B70" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C70" s="1"/>
-      <c r="D70" t="s">
-        <v>135</v>
-      </c>
       <c r="F70" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.2">
@@ -2013,7 +2040,7 @@
         <v>61</v>
       </c>
       <c r="B71" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C71" s="1"/>
       <c r="F71" t="s">
@@ -2025,7 +2052,7 @@
         <v>61</v>
       </c>
       <c r="B72" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C72" s="1"/>
       <c r="F72" t="s">
@@ -2037,7 +2064,7 @@
         <v>61</v>
       </c>
       <c r="B73" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C73" s="1"/>
       <c r="F73" t="s">
@@ -2049,7 +2076,7 @@
         <v>61</v>
       </c>
       <c r="B74" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C74" s="1"/>
       <c r="F74" t="s">
@@ -2061,7 +2088,7 @@
         <v>61</v>
       </c>
       <c r="B75" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C75" s="1"/>
       <c r="F75" t="s">
@@ -2072,20 +2099,23 @@
       <c r="A76" t="s">
         <v>61</v>
       </c>
-      <c r="B76" t="s">
-        <v>82</v>
+      <c r="B76" s="4" t="s">
+        <v>83</v>
       </c>
       <c r="C76" s="1"/>
+      <c r="D76" t="s">
+        <v>135</v>
+      </c>
       <c r="F76" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>61</v>
       </c>
-      <c r="B77" t="s">
-        <v>83</v>
+      <c r="B77" s="4" t="s">
+        <v>84</v>
       </c>
       <c r="C77" s="1"/>
       <c r="D77" t="s">
@@ -2099,8 +2129,8 @@
       <c r="A78" t="s">
         <v>61</v>
       </c>
-      <c r="B78" t="s">
-        <v>84</v>
+      <c r="B78" s="4" t="s">
+        <v>85</v>
       </c>
       <c r="C78" s="1"/>
       <c r="D78" t="s">
@@ -2115,14 +2145,11 @@
         <v>61</v>
       </c>
       <c r="B79" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C79" s="1"/>
-      <c r="D79" t="s">
-        <v>135</v>
-      </c>
       <c r="F79" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.2">
@@ -2130,7 +2157,7 @@
         <v>61</v>
       </c>
       <c r="B80" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C80" s="1"/>
       <c r="F80" t="s">
@@ -2142,7 +2169,7 @@
         <v>61</v>
       </c>
       <c r="B81" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C81" s="1"/>
       <c r="F81" t="s">
@@ -2151,12 +2178,18 @@
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
-        <v>61</v>
+        <v>116</v>
       </c>
       <c r="B82" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C82" s="1"/>
+      <c r="D82" t="s">
+        <v>136</v>
+      </c>
+      <c r="E82" t="s">
+        <v>149</v>
+      </c>
       <c r="F82" t="s">
         <v>126</v>
       </c>
@@ -2166,14 +2199,14 @@
         <v>116</v>
       </c>
       <c r="B83" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C83" s="1"/>
       <c r="D83" t="s">
         <v>136</v>
       </c>
       <c r="E83" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="F83" t="s">
         <v>126</v>
@@ -2184,14 +2217,14 @@
         <v>116</v>
       </c>
       <c r="B84" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C84" s="1"/>
       <c r="D84" t="s">
         <v>136</v>
       </c>
       <c r="E84" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="F84" t="s">
         <v>126</v>
@@ -2202,14 +2235,14 @@
         <v>116</v>
       </c>
       <c r="B85" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C85" s="1"/>
       <c r="D85" t="s">
         <v>136</v>
       </c>
       <c r="E85" t="s">
-        <v>151</v>
+        <v>141</v>
       </c>
       <c r="F85" t="s">
         <v>126</v>
@@ -2220,14 +2253,14 @@
         <v>116</v>
       </c>
       <c r="B86" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C86" s="1"/>
       <c r="D86" t="s">
         <v>136</v>
       </c>
       <c r="E86" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="F86" t="s">
         <v>126</v>
@@ -2238,14 +2271,14 @@
         <v>116</v>
       </c>
       <c r="B87" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C87" s="1"/>
       <c r="D87" t="s">
         <v>136</v>
       </c>
       <c r="E87" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="F87" t="s">
         <v>126</v>
@@ -2256,15 +2289,12 @@
         <v>116</v>
       </c>
       <c r="B88" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C88" s="1"/>
       <c r="D88" t="s">
         <v>136</v>
       </c>
-      <c r="E88" t="s">
-        <v>143</v>
-      </c>
       <c r="F88" t="s">
         <v>126</v>
       </c>
@@ -2274,11 +2304,11 @@
         <v>116</v>
       </c>
       <c r="B89" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C89" s="1"/>
       <c r="D89" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="F89" t="s">
         <v>126</v>
@@ -2289,11 +2319,11 @@
         <v>116</v>
       </c>
       <c r="B90" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C90" s="1"/>
       <c r="D90" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="F90" t="s">
         <v>126</v>
@@ -2304,11 +2334,14 @@
         <v>116</v>
       </c>
       <c r="B91" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C91" s="1"/>
       <c r="D91" t="s">
-        <v>136</v>
+        <v>138</v>
+      </c>
+      <c r="E91" t="s">
+        <v>152</v>
       </c>
       <c r="F91" t="s">
         <v>126</v>
@@ -2319,14 +2352,11 @@
         <v>116</v>
       </c>
       <c r="B92" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C92" s="1"/>
       <c r="D92" t="s">
-        <v>138</v>
-      </c>
-      <c r="E92" t="s">
-        <v>152</v>
+        <v>136</v>
       </c>
       <c r="F92" t="s">
         <v>126</v>
@@ -2337,7 +2367,7 @@
         <v>116</v>
       </c>
       <c r="B93" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C93" s="1"/>
       <c r="D93" t="s">
@@ -2352,12 +2382,15 @@
         <v>116</v>
       </c>
       <c r="B94" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C94" s="1"/>
       <c r="D94" t="s">
         <v>136</v>
       </c>
+      <c r="E94" t="s">
+        <v>144</v>
+      </c>
       <c r="F94" t="s">
         <v>126</v>
       </c>
@@ -2367,14 +2400,14 @@
         <v>116</v>
       </c>
       <c r="B95" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C95" s="1"/>
       <c r="D95" t="s">
         <v>136</v>
       </c>
       <c r="E95" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="F95" t="s">
         <v>126</v>
@@ -2385,14 +2418,14 @@
         <v>116</v>
       </c>
       <c r="B96" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C96" s="1"/>
       <c r="D96" t="s">
         <v>136</v>
       </c>
       <c r="E96" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="F96" t="s">
         <v>126</v>
@@ -2403,15 +2436,12 @@
         <v>116</v>
       </c>
       <c r="B97" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C97" s="1"/>
       <c r="D97" t="s">
         <v>136</v>
       </c>
-      <c r="E97" t="s">
-        <v>146</v>
-      </c>
       <c r="F97" t="s">
         <v>126</v>
       </c>
@@ -2421,11 +2451,11 @@
         <v>116</v>
       </c>
       <c r="B98" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C98" s="1"/>
       <c r="D98" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="F98" t="s">
         <v>126</v>
@@ -2436,11 +2466,11 @@
         <v>116</v>
       </c>
       <c r="B99" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C99" s="1"/>
       <c r="D99" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="F99" t="s">
         <v>126</v>
@@ -2451,11 +2481,14 @@
         <v>116</v>
       </c>
       <c r="B100" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C100" s="1"/>
       <c r="D100" t="s">
-        <v>136</v>
+        <v>138</v>
+      </c>
+      <c r="E100" t="s">
+        <v>153</v>
       </c>
       <c r="F100" t="s">
         <v>126</v>
@@ -2466,14 +2499,11 @@
         <v>116</v>
       </c>
       <c r="B101" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C101" s="1"/>
       <c r="D101" t="s">
-        <v>138</v>
-      </c>
-      <c r="E101" t="s">
-        <v>153</v>
+        <v>136</v>
       </c>
       <c r="F101" t="s">
         <v>126</v>
@@ -2484,7 +2514,7 @@
         <v>116</v>
       </c>
       <c r="B102" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C102" s="1"/>
       <c r="D102" t="s">
@@ -2499,12 +2529,15 @@
         <v>116</v>
       </c>
       <c r="B103" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C103" s="1"/>
       <c r="D103" t="s">
         <v>136</v>
       </c>
+      <c r="E103" t="s">
+        <v>143</v>
+      </c>
       <c r="F103" t="s">
         <v>126</v>
       </c>
@@ -2514,14 +2547,14 @@
         <v>116</v>
       </c>
       <c r="B104" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C104" s="1"/>
       <c r="D104" t="s">
         <v>136</v>
       </c>
       <c r="E104" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="F104" t="s">
         <v>126</v>
@@ -2532,14 +2565,14 @@
         <v>116</v>
       </c>
       <c r="B105" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C105" s="1"/>
       <c r="D105" t="s">
         <v>136</v>
       </c>
       <c r="E105" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F105" t="s">
         <v>126</v>
@@ -2550,14 +2583,11 @@
         <v>116</v>
       </c>
       <c r="B106" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C106" s="1"/>
       <c r="D106" t="s">
-        <v>136</v>
-      </c>
-      <c r="E106" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="F106" t="s">
         <v>126</v>
@@ -2568,11 +2598,11 @@
         <v>116</v>
       </c>
       <c r="B107" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C107" s="1"/>
       <c r="D107" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="F107" t="s">
         <v>126</v>
@@ -2583,7 +2613,7 @@
         <v>116</v>
       </c>
       <c r="B108" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C108" s="1"/>
       <c r="D108" t="s">
@@ -2595,20 +2625,28 @@
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
-        <v>116</v>
+        <v>27</v>
       </c>
       <c r="B109" t="s">
-        <v>115</v>
-      </c>
-      <c r="C109" s="1"/>
+        <v>29</v>
+      </c>
+      <c r="C109" t="s">
+        <v>31</v>
+      </c>
       <c r="D109" t="s">
-        <v>136</v>
+        <v>32</v>
+      </c>
+      <c r="E109" t="s">
+        <v>33</v>
       </c>
       <c r="F109" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:F109">
+    <sortCondition ref="A1:A109"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>

</xml_diff>